<commit_message>
chore: auto update fair data
</commit_message>
<xml_diff>
--- a/build/events_master.xlsx
+++ b/build/events_master.xlsx
@@ -634,7 +634,11 @@
       <c r="S2" t="n">
         <v>0.8</v>
       </c>
-      <c r="T2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -730,7 +734,11 @@
       <c r="S3" t="n">
         <v>0.8</v>
       </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -826,7 +834,11 @@
       <c r="S4" t="n">
         <v>0.8</v>
       </c>
-      <c r="T4" t="inlineStr"/>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -922,7 +934,11 @@
       <c r="S5" t="n">
         <v>0.8</v>
       </c>
-      <c r="T5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1018,7 +1034,11 @@
       <c r="S6" t="n">
         <v>0.8</v>
       </c>
-      <c r="T6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1114,7 +1134,11 @@
       <c r="S7" t="n">
         <v>0.8</v>
       </c>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1210,7 +1234,11 @@
       <c r="S8" t="n">
         <v>0.8</v>
       </c>
-      <c r="T8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1306,7 +1334,11 @@
       <c r="S9" t="n">
         <v>0.8</v>
       </c>
-      <c r="T9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1402,7 +1434,11 @@
       <c r="S10" t="n">
         <v>0.8</v>
       </c>
-      <c r="T10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1498,7 +1534,11 @@
       <c r="S11" t="n">
         <v>0.8</v>
       </c>
-      <c r="T11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1594,7 +1634,11 @@
       <c r="S12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1690,7 +1734,11 @@
       <c r="S13" t="n">
         <v>0.8</v>
       </c>
-      <c r="T13" t="inlineStr"/>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1786,7 +1834,11 @@
       <c r="S14" t="n">
         <v>0.8</v>
       </c>
-      <c r="T14" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1882,7 +1934,11 @@
       <c r="S15" t="n">
         <v>0.8</v>
       </c>
-      <c r="T15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1978,7 +2034,11 @@
       <c r="S16" t="n">
         <v>0.8</v>
       </c>
-      <c r="T16" t="inlineStr"/>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2074,7 +2134,11 @@
       <c r="S17" t="n">
         <v>0.8</v>
       </c>
-      <c r="T17" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2170,7 +2234,11 @@
       <c r="S18" t="n">
         <v>0.8</v>
       </c>
-      <c r="T18" t="inlineStr"/>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2266,7 +2334,11 @@
       <c r="S19" t="n">
         <v>0.8</v>
       </c>
-      <c r="T19" t="inlineStr"/>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2362,7 +2434,11 @@
       <c r="S20" t="n">
         <v>0.8</v>
       </c>
-      <c r="T20" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2458,7 +2534,11 @@
       <c r="S21" t="n">
         <v>0.8</v>
       </c>
-      <c r="T21" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2554,7 +2634,11 @@
       <c r="S22" t="n">
         <v>0.8</v>
       </c>
-      <c r="T22" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2650,7 +2734,11 @@
       <c r="S23" t="n">
         <v>0.8</v>
       </c>
-      <c r="T23" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2746,7 +2834,11 @@
       <c r="S24" t="n">
         <v>0.8</v>
       </c>
-      <c r="T24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2842,7 +2934,11 @@
       <c r="S25" t="n">
         <v>0.8</v>
       </c>
-      <c r="T25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2938,7 +3034,11 @@
       <c r="S26" t="n">
         <v>0.8</v>
       </c>
-      <c r="T26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3034,7 +3134,11 @@
       <c r="S27" t="n">
         <v>0.8</v>
       </c>
-      <c r="T27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3130,7 +3234,11 @@
       <c r="S28" t="n">
         <v>0.8</v>
       </c>
-      <c r="T28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>2026-06-03T08:57:30+00:00</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>